<commit_message>
Record verified main upload and final WBS completion states
</commit_message>
<xml_diff>
--- a/docs/CultureBridge_WBS_세부기능_정리_2026-10-23.xlsx
+++ b/docs/CultureBridge_WBS_세부기능_정리_2026-10-23.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" r:id="R45317746f798428c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" r:id="Racd1fd9092d446c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20606,7 +20606,7 @@
         <x:v>김상엽</x:v>
       </x:c>
       <x:c r="G260" s="146" t="str">
-        <x:v>진행 중</x:v>
+        <x:v>완료</x:v>
       </x:c>
       <x:c r="H260" s="152"/>
       <x:c r="I260" s="149"/>

</xml_diff>